<commit_message>
Shift start dates in Plan_Group3_VoDuyBinh Excel sheets to start on July 13th
</commit_message>
<xml_diff>
--- a/Ebooks/Plan_Group3_VoDuyBinh.xlsx
+++ b/Ebooks/Plan_Group3_VoDuyBinh.xlsx
@@ -1279,11 +1279,11 @@
       </c>
       <c r="D4" s="8">
         <f>MIN(D5:D9)</f>
-        <v>46237</v>
+        <v>46218</v>
       </c>
       <c r="E4" s="8">
         <f>MAX(E5:E9)</f>
-        <v>46244</v>
+        <v>46225</v>
       </c>
       <c r="F4" s="2" t="str">
         <f t="shared" ref="F4:AK4" si="0">IF(AND(F$1&gt;=$D4,F$1&lt;=$E4),"█","")</f>
@@ -1530,11 +1530,11 @@
       </c>
       <c r="D5" s="11">
         <f>IF(C5&gt;0,INDEX(F$1:CB$1,MATCH("█",F5:CB5,0)),"")</f>
-        <v>46237</v>
+        <v>46218</v>
       </c>
       <c r="E5" s="11">
         <f>IF(C5&gt;0,INDEX(F$1:CB$1,MATCH("█",F5:CB5,0)+C5-1),"")</f>
-        <v>46238</v>
+        <v>46219</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>27</v>
@@ -1629,11 +1629,11 @@
       </c>
       <c r="D6" s="11">
         <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)),"")</f>
-        <v>46239</v>
+        <v>46220</v>
       </c>
       <c r="E6" s="11">
         <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)+C6-1),"")</f>
-        <v>46239</v>
+        <v>46220</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1726,11 +1726,11 @@
       </c>
       <c r="D7" s="11">
         <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)),"")</f>
-        <v>46240</v>
+        <v>46221</v>
       </c>
       <c r="E7" s="11">
         <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)+C7-1),"")</f>
-        <v>46241</v>
+        <v>46222</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1825,11 +1825,11 @@
       </c>
       <c r="D8" s="11">
         <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)),"")</f>
-        <v>46244</v>
+        <v>46225</v>
       </c>
       <c r="E8" s="11">
         <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)+C8-1),"")</f>
-        <v>46244</v>
+        <v>46225</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1922,11 +1922,11 @@
       </c>
       <c r="D9" s="11">
         <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)),"")</f>
-        <v>46240</v>
+        <v>46221</v>
       </c>
       <c r="E9" s="11">
         <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)+C9-1),"")</f>
-        <v>46244</v>
+        <v>46225</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -2023,11 +2023,11 @@
       </c>
       <c r="D10" s="8">
         <f>MIN(D11:D13)</f>
-        <v>46245</v>
+        <v>46226</v>
       </c>
       <c r="E10" s="8">
         <f>MAX(E11:E13)</f>
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="F10" s="2">
         <f t="shared" ref="F10:AK10" si="3">IF(AND(F$1&gt;=$D10,F$1&lt;=$E10),"█","")</f>
@@ -2272,11 +2272,11 @@
       </c>
       <c r="D11" s="11">
         <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)),"")</f>
-        <v>46245</v>
+        <v>46226</v>
       </c>
       <c r="E11" s="11">
         <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)+C11-1),"")</f>
-        <v>46245</v>
+        <v>46226</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
@@ -2369,11 +2369,11 @@
       </c>
       <c r="D12" s="11">
         <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)),"")</f>
-        <v>46246</v>
+        <v>46227</v>
       </c>
       <c r="E12" s="11">
         <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)+C12-1),"")</f>
-        <v>46247</v>
+        <v>46228</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
@@ -2468,11 +2468,11 @@
       </c>
       <c r="D13" s="11">
         <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)),"")</f>
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="E13" s="11">
         <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)+C13-1),"")</f>
-        <v>46248</v>
+        <v>46229</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -2565,11 +2565,11 @@
       </c>
       <c r="D14" s="11">
         <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)),"")</f>
-        <v>46251</v>
+        <v>46232</v>
       </c>
       <c r="E14" s="11">
         <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)+C14-1),"")</f>
-        <v>46255</v>
+        <v>46236</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
@@ -2670,11 +2670,11 @@
       </c>
       <c r="D15" s="8">
         <f>MIN(D16:D23)</f>
-        <v>46258</v>
+        <v>46239</v>
       </c>
       <c r="E15" s="8">
         <f>MAX(E16:E23)</f>
-        <v>46297</v>
+        <v>46278</v>
       </c>
       <c r="F15" s="2">
         <f t="shared" ref="F15:AK15" si="6">IF(AND(F$1&gt;=$D15,F$1&lt;=$E15),"█","")</f>
@@ -2945,11 +2945,11 @@
       </c>
       <c r="D16" s="11">
         <f t="shared" ref="D16:D25" si="10">IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)),"")</f>
-        <v>46258</v>
+        <v>46239</v>
       </c>
       <c r="E16" s="11">
         <f t="shared" ref="E16:E25" si="11">IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)+C16-1),"")</f>
-        <v>46260</v>
+        <v>46241</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -3046,11 +3046,11 @@
       </c>
       <c r="D17" s="11">
         <f t="shared" si="10"/>
-        <v>46261</v>
+        <v>46242</v>
       </c>
       <c r="E17" s="11">
         <f t="shared" si="11"/>
-        <v>46262</v>
+        <v>46243</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -3145,11 +3145,11 @@
       </c>
       <c r="D18" s="11">
         <f t="shared" si="10"/>
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="E18" s="11">
         <f t="shared" si="11"/>
-        <v>46268</v>
+        <v>46249</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -3248,11 +3248,11 @@
       </c>
       <c r="D19" s="11">
         <f t="shared" si="10"/>
-        <v>46265</v>
+        <v>46246</v>
       </c>
       <c r="E19" s="11">
         <f t="shared" si="11"/>
-        <v>46269</v>
+        <v>46250</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -3353,11 +3353,11 @@
       </c>
       <c r="D20" s="11">
         <f t="shared" si="10"/>
-        <v>46272</v>
+        <v>46253</v>
       </c>
       <c r="E20" s="11">
         <f t="shared" si="11"/>
-        <v>46286</v>
+        <v>46267</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -3470,11 +3470,11 @@
       </c>
       <c r="D21" s="11">
         <f t="shared" si="10"/>
-        <v>46287</v>
+        <v>46268</v>
       </c>
       <c r="E21" s="11">
         <f t="shared" si="11"/>
-        <v>46290</v>
+        <v>46271</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -3573,11 +3573,11 @@
       </c>
       <c r="D22" s="11">
         <f t="shared" si="10"/>
-        <v>46293</v>
+        <v>46274</v>
       </c>
       <c r="E22" s="11">
         <f t="shared" si="11"/>
-        <v>46295</v>
+        <v>46276</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -3674,11 +3674,11 @@
       </c>
       <c r="D23" s="11">
         <f t="shared" si="10"/>
-        <v>46296</v>
+        <v>46277</v>
       </c>
       <c r="E23" s="11">
         <f t="shared" si="11"/>
-        <v>46297</v>
+        <v>46278</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -3773,11 +3773,11 @@
       </c>
       <c r="D24" s="11">
         <f t="shared" si="10"/>
-        <v>46245</v>
+        <v>46226</v>
       </c>
       <c r="E24" s="11">
         <f t="shared" si="11"/>
-        <v>46293</v>
+        <v>46274</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -3938,11 +3938,11 @@
       </c>
       <c r="D25" s="11">
         <f t="shared" si="10"/>
-        <v>46300</v>
+        <v>46281</v>
       </c>
       <c r="E25" s="11">
         <f t="shared" si="11"/>
-        <v>46302</v>
+        <v>46283</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>

</xml_diff>